<commit_message>
Update FDR correction procedure
</commit_message>
<xml_diff>
--- a/figures/supplementary/Raw-p-val_FDR_corrected.xlsx
+++ b/figures/supplementary/Raw-p-val_FDR_corrected.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,20 +459,10 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Stats.1</t>
+          <t>FDR_BH_pvalue</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>p-value.1</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>FDR_BH_pvalue</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>FDR_BH_significant_0.05</t>
         </is>
@@ -502,17 +492,19 @@
       <c r="E2" t="n">
         <v>1.772e-66</v>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="n">
+      <c r="F2" t="n">
         <v>5.6704e-65</v>
       </c>
-      <c r="I2" t="b">
+      <c r="G2" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2A</t>
+        </is>
+      </c>
       <c r="B3" t="inlineStr">
         <is>
           <t>Y2H</t>
@@ -531,12 +523,10 @@
       <c r="E3" t="n">
         <v>0.3379</v>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="n">
+      <c r="F3" t="n">
         <v>0.6007111111111111</v>
       </c>
-      <c r="I3" t="b">
+      <c r="G3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -564,17 +554,19 @@
       <c r="E4" t="n">
         <v>8.586e-38</v>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="n">
+      <c r="F4" t="n">
         <v>1.37376e-36</v>
       </c>
-      <c r="I4" t="b">
+      <c r="G4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2B</t>
+        </is>
+      </c>
       <c r="B5" t="inlineStr">
         <is>
           <t>Y2H</t>
@@ -593,12 +585,10 @@
       <c r="E5" t="n">
         <v>0.9976</v>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I5" t="b">
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -626,12 +616,10 @@
       <c r="E6" t="n">
         <v>7.298e-16</v>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="n">
+      <c r="F6" t="n">
         <v>4.67072e-15</v>
       </c>
-      <c r="I6" t="b">
+      <c r="G6" t="n">
         <v>1</v>
       </c>
     </row>
@@ -659,12 +647,10 @@
       <c r="E7" t="n">
         <v>2.995e-14</v>
       </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="n">
+      <c r="F7" t="n">
         <v>1.597333333333333e-13</v>
       </c>
-      <c r="I7" t="b">
+      <c r="G7" t="n">
         <v>1</v>
       </c>
     </row>
@@ -692,12 +678,10 @@
       <c r="E8" t="n">
         <v>3.996e-17</v>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="n">
+      <c r="F8" t="n">
         <v>3.1968e-16</v>
       </c>
-      <c r="I8" t="b">
+      <c r="G8" t="n">
         <v>1</v>
       </c>
     </row>
@@ -725,12 +709,10 @@
       <c r="E9" t="n">
         <v>3.531e-28</v>
       </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="n">
+      <c r="F9" t="n">
         <v>3.7664e-27</v>
       </c>
-      <c r="I9" t="b">
+      <c r="G9" t="n">
         <v>1</v>
       </c>
     </row>
@@ -758,12 +740,10 @@
       <c r="E10" t="n">
         <v>0.001</v>
       </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="n">
+      <c r="F10" t="n">
         <v>0.002461538461538462</v>
       </c>
-      <c r="I10" t="b">
+      <c r="G10" t="n">
         <v>1</v>
       </c>
     </row>
@@ -791,12 +771,10 @@
       <c r="E11" t="n">
         <v>0.99</v>
       </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="n">
-        <v>1</v>
-      </c>
-      <c r="I11" t="b">
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -824,12 +802,10 @@
       <c r="E12" t="n">
         <v>1</v>
       </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I12" t="b">
+      <c r="F12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" t="n">
         <v>0</v>
       </c>
     </row>
@@ -857,12 +833,10 @@
       <c r="E13" t="n">
         <v>1</v>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="n">
-        <v>1</v>
-      </c>
-      <c r="I13" t="b">
+      <c r="F13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" t="n">
         <v>0</v>
       </c>
     </row>
@@ -890,12 +864,10 @@
       <c r="E14" t="n">
         <v>0.00022</v>
       </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="n">
+      <c r="F14" t="n">
         <v>0.0007040000000000001</v>
       </c>
-      <c r="I14" t="b">
+      <c r="G14" t="n">
         <v>1</v>
       </c>
     </row>
@@ -923,12 +895,10 @@
       <c r="E15" t="n">
         <v>1.106e-08</v>
       </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="n">
+      <c r="F15" t="n">
         <v>5.056e-08</v>
       </c>
-      <c r="I15" t="b">
+      <c r="G15" t="n">
         <v>1</v>
       </c>
     </row>
@@ -956,12 +926,10 @@
       <c r="E16" t="n">
         <v>9.670999999999999e-06</v>
       </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="n">
+      <c r="F16" t="n">
         <v>3.8684e-05</v>
       </c>
-      <c r="I16" t="b">
+      <c r="G16" t="n">
         <v>1</v>
       </c>
     </row>
@@ -989,17 +957,19 @@
       <c r="E17" t="n">
         <v>0.107</v>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="n">
+      <c r="F17" t="n">
         <v>0.214</v>
       </c>
-      <c r="I17" t="b">
+      <c r="G17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr"/>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>6C</t>
+        </is>
+      </c>
       <c r="B18" t="inlineStr">
         <is>
           <t>AE-MS</t>
@@ -1018,17 +988,19 @@
       <c r="E18" t="n">
         <v>0.000454</v>
       </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="n">
+      <c r="F18" t="n">
         <v>0.001210666666666667</v>
       </c>
-      <c r="I18" t="b">
+      <c r="G18" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>6C</t>
+        </is>
+      </c>
       <c r="B19" t="inlineStr">
         <is>
           <t>AE-MS</t>
@@ -1047,17 +1019,19 @@
       <c r="E19" t="n">
         <v>0.0414</v>
       </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="n">
+      <c r="F19" t="n">
         <v>0.08832</v>
       </c>
-      <c r="I19" t="b">
+      <c r="G19" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>6C</t>
+        </is>
+      </c>
       <c r="B20" t="inlineStr">
         <is>
           <t>AE-MS</t>
@@ -1076,12 +1050,10 @@
       <c r="E20" t="n">
         <v>0.000275</v>
       </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="n">
+      <c r="F20" t="n">
         <v>0.0008</v>
       </c>
-      <c r="I20" t="b">
+      <c r="G20" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1109,12 +1081,10 @@
       <c r="E21" t="n">
         <v>0.9825</v>
       </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="n">
-        <v>1</v>
-      </c>
-      <c r="I21" t="b">
+      <c r="F21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1142,12 +1112,10 @@
       <c r="E22" t="n">
         <v>0.9917</v>
       </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="n">
-        <v>1</v>
-      </c>
-      <c r="I22" t="b">
+      <c r="F22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1175,12 +1143,10 @@
       <c r="E23" t="n">
         <v>0.8502999999999999</v>
       </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="n">
-        <v>1</v>
-      </c>
-      <c r="I23" t="b">
+      <c r="F23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1208,12 +1174,10 @@
       <c r="E24" t="n">
         <v>0.0002098</v>
       </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="n">
+      <c r="F24" t="n">
         <v>0.0007040000000000001</v>
       </c>
-      <c r="I24" t="b">
+      <c r="G24" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1241,12 +1205,10 @@
       <c r="E25" t="n">
         <v>0.9845</v>
       </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="n">
-        <v>1</v>
-      </c>
-      <c r="I25" t="b">
+      <c r="F25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1274,12 +1236,10 @@
       <c r="E26" t="n">
         <v>0.9972</v>
       </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="n">
-        <v>1</v>
-      </c>
-      <c r="I26" t="b">
+      <c r="F26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1307,12 +1267,10 @@
       <c r="E27" t="n">
         <v>0.9643</v>
       </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="n">
-        <v>1</v>
-      </c>
-      <c r="I27" t="b">
+      <c r="F27" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1340,12 +1298,10 @@
       <c r="E28" t="n">
         <v>0.5155</v>
       </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="n">
+      <c r="F28" t="n">
         <v>0.8248</v>
       </c>
-      <c r="I28" t="b">
+      <c r="G28" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1373,12 +1329,10 @@
       <c r="E29" t="n">
         <v>0.7</v>
       </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="n">
-        <v>1</v>
-      </c>
-      <c r="I29" t="b">
+      <c r="F29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1406,12 +1360,10 @@
       <c r="E30" t="n">
         <v>0.27</v>
       </c>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="n">
+      <c r="F30" t="n">
         <v>0.5082352941176471</v>
       </c>
-      <c r="I30" t="b">
+      <c r="G30" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1439,12 +1391,10 @@
       <c r="E31" t="n">
         <v>0.37</v>
       </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="n">
+      <c r="F31" t="n">
         <v>0.623157894736842</v>
       </c>
-      <c r="I31" t="b">
+      <c r="G31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1472,12 +1422,10 @@
       <c r="E32" t="n">
         <v>0.038</v>
       </c>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="n">
+      <c r="F32" t="n">
         <v>0.08685714285714285</v>
       </c>
-      <c r="I32" t="b">
+      <c r="G32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1505,12 +1453,10 @@
       <c r="E33" t="n">
         <v>0.96</v>
       </c>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="n">
-        <v>1</v>
-      </c>
-      <c r="I33" t="b">
+      <c r="F33" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1592,12 +1538,16 @@
       <c r="F2" t="n">
         <v>3.568e-13</v>
       </c>
-      <c r="G2" t="b">
+      <c r="G2" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2C</t>
+        </is>
+      </c>
       <c r="B3" t="inlineStr">
         <is>
           <t>Y2H</t>
@@ -1619,7 +1569,7 @@
       <c r="F3" t="n">
         <v>0.002887</v>
       </c>
-      <c r="G3" t="b">
+      <c r="G3" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1650,7 +1600,7 @@
       <c r="F4" t="n">
         <v>1.1704e-13</v>
       </c>
-      <c r="G4" t="b">
+      <c r="G4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1681,7 +1631,7 @@
       <c r="F5" t="n">
         <v>2.352e-06</v>
       </c>
-      <c r="G5" t="b">
+      <c r="G5" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1696,7 +1646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1727,20 +1677,10 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Stats.1</t>
+          <t>FDR_BH_pvalue</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>p-value.1</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>FDR_BH_pvalue</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>FDR_BH_significant_0.05</t>
         </is>
@@ -1770,17 +1710,19 @@
       <c r="E2" t="n">
         <v>8.407e-32</v>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="n">
+      <c r="F2" t="n">
         <v>1.84954e-30</v>
       </c>
-      <c r="I2" t="b">
+      <c r="G2" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2D</t>
+        </is>
+      </c>
       <c r="B3" t="inlineStr">
         <is>
           <t>Y2H</t>
@@ -1799,12 +1741,10 @@
       <c r="E3" t="n">
         <v>0.6906</v>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="n">
+      <c r="F3" t="n">
         <v>0.9996</v>
       </c>
-      <c r="I3" t="b">
+      <c r="G3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1832,17 +1772,19 @@
       <c r="E4" t="n">
         <v>0.05691</v>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="n">
+      <c r="F4" t="n">
         <v>0.6260100000000001</v>
       </c>
-      <c r="I4" t="b">
+      <c r="G4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2E</t>
+        </is>
+      </c>
       <c r="B5" t="inlineStr">
         <is>
           <t>Y2H</t>
@@ -1861,12 +1803,10 @@
       <c r="E5" t="n">
         <v>0.9901</v>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="n">
+      <c r="F5" t="n">
         <v>0.9996</v>
       </c>
-      <c r="I5" t="b">
+      <c r="G5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1894,12 +1834,10 @@
       <c r="E6" t="n">
         <v>0.9937</v>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="n">
+      <c r="F6" t="n">
         <v>0.9996</v>
       </c>
-      <c r="I6" t="b">
+      <c r="G6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1927,12 +1865,10 @@
       <c r="E7" t="n">
         <v>0.9972</v>
       </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="n">
+      <c r="F7" t="n">
         <v>0.9996</v>
       </c>
-      <c r="I7" t="b">
+      <c r="G7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1960,12 +1896,10 @@
       <c r="E8" t="n">
         <v>0.9996</v>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="n">
+      <c r="F8" t="n">
         <v>0.9996</v>
       </c>
-      <c r="I8" t="b">
+      <c r="G8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1993,12 +1927,10 @@
       <c r="E9" t="n">
         <v>0.9801</v>
       </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="n">
+      <c r="F9" t="n">
         <v>0.9996</v>
       </c>
-      <c r="I9" t="b">
+      <c r="G9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2026,12 +1958,10 @@
       <c r="E10" t="n">
         <v>0.583</v>
       </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="n">
+      <c r="F10" t="n">
         <v>0.9996</v>
       </c>
-      <c r="I10" t="b">
+      <c r="G10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2059,12 +1989,10 @@
       <c r="E11" t="n">
         <v>0.8456</v>
       </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="n">
+      <c r="F11" t="n">
         <v>0.9996</v>
       </c>
-      <c r="I11" t="b">
+      <c r="G11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2092,12 +2020,10 @@
       <c r="E12" t="n">
         <v>0.3647</v>
       </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="n">
+      <c r="F12" t="n">
         <v>0.9996</v>
       </c>
-      <c r="I12" t="b">
+      <c r="G12" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2125,12 +2051,10 @@
       <c r="E13" t="n">
         <v>0.5553</v>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="n">
+      <c r="F13" t="n">
         <v>0.9996</v>
       </c>
-      <c r="I13" t="b">
+      <c r="G13" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2158,12 +2082,10 @@
       <c r="E14" t="n">
         <v>0.37</v>
       </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
-      <c r="H14" t="n">
+      <c r="F14" t="n">
         <v>0.9996</v>
       </c>
-      <c r="I14" t="b">
+      <c r="G14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2191,12 +2113,10 @@
       <c r="E15" t="n">
         <v>0.6</v>
       </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="n">
+      <c r="F15" t="n">
         <v>0.9996</v>
       </c>
-      <c r="I15" t="b">
+      <c r="G15" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2224,12 +2144,10 @@
       <c r="E16" t="n">
         <v>0.87</v>
       </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="n">
+      <c r="F16" t="n">
         <v>0.9996</v>
       </c>
-      <c r="I16" t="b">
+      <c r="G16" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2257,12 +2175,10 @@
       <c r="E17" t="n">
         <v>0.34</v>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="n">
+      <c r="F17" t="n">
         <v>0.9996</v>
       </c>
-      <c r="I17" t="b">
+      <c r="G17" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2290,12 +2206,10 @@
       <c r="E18" t="n">
         <v>0.87</v>
       </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="n">
+      <c r="F18" t="n">
         <v>0.9996</v>
       </c>
-      <c r="I18" t="b">
+      <c r="G18" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2323,12 +2237,10 @@
       <c r="E19" t="n">
         <v>0.96</v>
       </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="n">
+      <c r="F19" t="n">
         <v>0.9996</v>
       </c>
-      <c r="I19" t="b">
+      <c r="G19" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2356,12 +2268,10 @@
       <c r="E20" t="n">
         <v>0.36</v>
       </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="n">
+      <c r="F20" t="n">
         <v>0.9996</v>
       </c>
-      <c r="I20" t="b">
+      <c r="G20" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2389,12 +2299,10 @@
       <c r="E21" t="n">
         <v>0.24</v>
       </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="n">
+      <c r="F21" t="n">
         <v>0.9996</v>
       </c>
-      <c r="I21" t="b">
+      <c r="G21" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2422,12 +2330,10 @@
       <c r="E22" t="n">
         <v>0.17</v>
       </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="n">
+      <c r="F22" t="n">
         <v>0.9996</v>
       </c>
-      <c r="I22" t="b">
+      <c r="G22" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2455,12 +2361,10 @@
       <c r="E23" t="n">
         <v>0.7</v>
       </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="n">
+      <c r="F23" t="n">
         <v>0.9996</v>
       </c>
-      <c r="I23" t="b">
+      <c r="G23" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2542,12 +2446,16 @@
       <c r="F2" t="n">
         <v>1.665e-07</v>
       </c>
-      <c r="G2" t="b">
+      <c r="G2" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2F</t>
+        </is>
+      </c>
       <c r="B3" t="inlineStr">
         <is>
           <t>Y2H</t>
@@ -2569,7 +2477,7 @@
       <c r="F3" t="n">
         <v>0.002058</v>
       </c>
-      <c r="G3" t="b">
+      <c r="G3" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>